<commit_message>
API key error fixed
</commit_message>
<xml_diff>
--- a/voxreach_ai/sample_customers.xlsx
+++ b/voxreach_ai/sample_customers.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>name</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Request for a Demo of CRM</t>
   </si>
   <si>
-    <t>Rahul</t>
-  </si>
-  <si>
     <t/>
   </si>
 </sst>
@@ -60,14 +57,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -523,148 +513,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1046,30 +1036,19 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>9999999999</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="4" spans="3:3">
       <c r="C4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:2">
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>